<commit_message>
Renomeia coluna Tipo para TipoEquipamento
O SharePoint em português já tem uma coluna interna chamada Tipo, então
o nome não pode ser usado na lista Equipamentos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XH4MAt6mPYqdihLEh8FYnK
</commit_message>
<xml_diff>
--- a/controle-calibracao-qr/1-sharepoint/modelo-equipamentos.xlsx
+++ b/controle-calibracao-qr/1-sharepoint/modelo-equipamentos.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -92,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -101,9 +100,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +498,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>TipoEquipamento</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -629,10 +629,10 @@
       <c r="G3" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="7" t="n">
         <v>46487</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -672,10 +672,10 @@
       <c r="G4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="7" t="n">
         <v>46147</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="7" t="n">
         <v>46331</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -715,10 +715,10 @@
       <c r="G5" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="7" t="n">
         <v>45870</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="7" t="n">
         <v>46235</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -758,10 +758,10 @@
       <c r="G6" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="7" t="n">
         <v>46188</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="7" t="n">
         <v>46553</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -801,10 +801,10 @@
       <c r="G7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="7" t="n">
         <v>46162</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="7" t="n">
         <v>46346</v>
       </c>
       <c r="J7" s="3" t="inlineStr">

</xml_diff>